<commit_message>
Evaluation results and code updates
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,67 +474,155 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Qwen 2.5 72B</t>
+          <t>Qwen 2.5 7B - ZeroShot</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.387</v>
+        <v>1.785</v>
       </c>
       <c r="C3" t="n">
-        <v>1.248</v>
+        <v>1.234</v>
       </c>
       <c r="D3" t="n">
-        <v>0.188</v>
+        <v>0.14</v>
       </c>
       <c r="E3" t="n">
-        <v>0.392</v>
+        <v>0.381</v>
       </c>
       <c r="F3" t="n">
-        <v>0.178</v>
+        <v>0.133</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Llama 3 8B</t>
+          <t>Qwen 2.5 72B</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.383</v>
+        <v>1.387</v>
       </c>
       <c r="C4" t="n">
-        <v>2.229</v>
+        <v>1.248</v>
       </c>
       <c r="D4" t="n">
-        <v>0.154</v>
+        <v>0.188</v>
       </c>
       <c r="E4" t="n">
-        <v>0.326</v>
+        <v>0.392</v>
       </c>
       <c r="F4" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.178</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Qwen 2.5 72B - ZeroShot</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.392</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.254</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.164</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Llama 3 8B</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.383</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.229</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Llama 3 8B - ZeroShot</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1.857</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2.246</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Llama 3 70B</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B8" t="n">
         <v>1.81</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C8" t="n">
         <v>2.02</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D8" t="n">
         <v>0.208</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E8" t="n">
         <v>0.407</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F8" t="n">
         <v>0.182</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Llama 3 70B - ZeroShot</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1.711</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.999</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.228</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.163</v>
       </c>
     </row>
   </sheetData>
@@ -548,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,58 +707,134 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Qwen 2.5 72B</t>
+          <t>Qwen 2.5 7B - ZeroShot</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>426</v>
+        <v>551</v>
       </c>
       <c r="C4" t="n">
-        <v>195</v>
+        <v>352</v>
       </c>
       <c r="D4" t="n">
-        <v>249</v>
+        <v>58</v>
       </c>
       <c r="E4" t="n">
-        <v>130</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Llama 3 8B</t>
+          <t>Qwen 2.5 72B</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>765</v>
+        <v>426</v>
       </c>
       <c r="C5" t="n">
-        <v>71</v>
+        <v>195</v>
       </c>
       <c r="D5" t="n">
-        <v>160</v>
+        <v>249</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Qwen 2.5 72B - ZeroShot</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>453</v>
+      </c>
+      <c r="C6" t="n">
+        <v>273</v>
+      </c>
+      <c r="D6" t="n">
+        <v>172</v>
+      </c>
+      <c r="E6" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Llama 3 8B</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>765</v>
+      </c>
+      <c r="C7" t="n">
+        <v>71</v>
+      </c>
+      <c r="D7" t="n">
+        <v>160</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Llama 3 8B - ZeroShot</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>872</v>
+      </c>
+      <c r="C8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D8" t="n">
+        <v>96</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Llama 3 70B</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B9" t="n">
         <v>444</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C9" t="n">
         <v>239</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D9" t="n">
         <v>226</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E9" t="n">
         <v>91</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Llama 3 70B - ZeroShot</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>488</v>
+      </c>
+      <c r="C10" t="n">
+        <v>228</v>
+      </c>
+      <c r="D10" t="n">
+        <v>228</v>
+      </c>
+      <c r="E10" t="n">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Load ground truth only for the 1000 songs under evaluation
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -673,16 +673,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>647</v>
+        <v>368</v>
       </c>
       <c r="C2" t="n">
-        <v>240</v>
+        <v>150</v>
       </c>
       <c r="D2" t="n">
-        <v>229</v>
+        <v>98</v>
       </c>
       <c r="E2" t="n">
-        <v>686</v>
+        <v>384</v>
       </c>
     </row>
     <row r="3">

</xml_diff>